<commit_message>
feat: selesai Tahap C Modul Inbound (Receiving & Put-away)
</commit_message>
<xml_diff>
--- a/Roadmap Backend WMS SaaS.xlsx
+++ b/Roadmap Backend WMS SaaS.xlsx
@@ -49,16 +49,16 @@
     <t>B1. API Manajemen Produk (Tambah, Edit, Hapus kategori Raw Material, Finished Good, dll) .+1B2. API Manajemen Gudang &amp; Setting (Tipe Gudang, Metode FIFO/FEFO/LIFO) .B3. API Manajemen Lokasi (Generate Racking &amp; Palleting).+1</t>
   </si>
   <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>Modul Inbound (Masuk)</t>
+  </si>
+  <si>
+    <t>C1. Endpoint POST /api/v1/receiving (Merekam barang datang dari supplier) .C2. Endpoint POST /api/v1/put-away (Menempatkan barang ke rak/lokasi spesifik &amp; catat ke tabel InventoryBatch).</t>
+  </si>
+  <si>
     <t>false</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>Modul Inbound (Masuk)</t>
-  </si>
-  <si>
-    <t>C1. Endpoint POST /api/v1/receiving (Merekam barang datang dari supplier) .C2. Endpoint POST /api/v1/put-away (Menempatkan barang ke rak/lokasi spesifik &amp; catat ke tabel InventoryBatch).</t>
   </si>
   <si>
     <t>D</t>
@@ -524,21 +524,21 @@
         <v>10</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="31.5">
       <c r="A4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="31.5">
@@ -552,7 +552,7 @@
         <v>17</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="45">
@@ -566,7 +566,7 @@
         <v>20</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="32.25">
@@ -580,7 +580,7 @@
         <v>23</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: complete WMS core modules (Storage, Outbound, and Dashboard Analytics)
</commit_message>
<xml_diff>
--- a/Roadmap Backend WMS SaaS.xlsx
+++ b/Roadmap Backend WMS SaaS.xlsx
@@ -58,25 +58,25 @@
     <t>C1. Endpoint POST /api/v1/receiving (Merekam barang datang dari supplier) .C2. Endpoint POST /api/v1/put-away (Menempatkan barang ke rak/lokasi spesifik &amp; catat ke tabel InventoryBatch).</t>
   </si>
   <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Modul Storage (Inventori)</t>
+  </si>
+  <si>
+    <t>D1. Endpoint GET /api/v1/storage/stock (Menampilkan total stok barang real-time per lokasi) .D2. Endpoint POST /api/v1/storage/opname (Mencatat hasil Stock Opname fisik vs sistem).</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>Modul Outbound (Keluar)</t>
+  </si>
+  <si>
+    <t>E1. Endpoint GET /api/v1/order/check (Validasi ketersediaan stok sebelum dikirim) .E2. Endpoint POST /api/v1/order/pick (Logika Inti: Mengambil barang dari InventoryBatch menggunakan aturan FIFO/FEFO/LIFO) .E3. Endpoint POST /api/v1/shipment (Update status pengiriman &amp; log transaksi).</t>
+  </si>
+  <si>
     <t>false</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>Modul Storage (Inventori)</t>
-  </si>
-  <si>
-    <t>D1. Endpoint GET /api/v1/storage/stock (Menampilkan total stok barang real-time per lokasi) .D2. Endpoint POST /api/v1/storage/opname (Mencatat hasil Stock Opname fisik vs sistem).</t>
-  </si>
-  <si>
-    <t>E</t>
-  </si>
-  <si>
-    <t>Modul Outbound (Keluar)</t>
-  </si>
-  <si>
-    <t>E1. Endpoint GET /api/v1/order/check (Validasi ketersediaan stok sebelum dikirim) .E2. Endpoint POST /api/v1/order/pick (Logika Inti: Mengambil barang dari InventoryBatch menggunakan aturan FIFO/FEFO/LIFO) .E3. Endpoint POST /api/v1/shipment (Update status pengiriman &amp; log transaksi).</t>
   </si>
   <si>
     <t>F</t>
@@ -538,35 +538,35 @@
         <v>13</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="31.5">
       <c r="A5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="D5" s="3" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="45">
       <c r="A6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>14</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="32.25">
@@ -580,7 +580,7 @@
         <v>23</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>